<commit_message>
CVE remediation summary 2026-08-12
</commit_message>
<xml_diff>
--- a/namespace/res-tmp/ticket_preview_2026-08-12.xlsx
+++ b/namespace/res-tmp/ticket_preview_2026-08-12.xlsx
@@ -483,7 +483,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rafay</t>
+          <t>(blank)</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -609,11 +609,6 @@
           <t>v1.42.0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>rafay</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Critical</t>
@@ -639,7 +634,7 @@
           <t>CVE-KEY: CVE-2026-53713|calico/operator|v1.42.0
 Severity: Critical
 Image: calico/operator:v1.42.0
-Namespace: rafay
+Namespace: unmapped
 First seen: 2026-07-20
 Due: 2026-08-19
 Reference: https://harbor-registry.dev.rafay-edge.net/harbor/projects/3/repositories/calico%2Foperator/artifacts-tab/artifacts/sha256:23c9bacd1ed01cd585372032c5b494ceee9a1c7e7f66d3d158c2146a2e8c0118</t>
@@ -667,11 +662,6 @@
           <t>1.2.16-6</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>rafay</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Critical</t>
@@ -697,7 +687,7 @@
           <t>CVE-KEY: CVE-2026-34182|helm-exporter|1.2.16-6
 Severity: Critical
 Image: helm-exporter:1.2.16-6
-Namespace: rafay
+Namespace: unmapped
 First seen: 2026-06-11
 Due: 2026-08-19
 Reference: https://harbor-registry.dev.rafay-edge.net/harbor/projects/3/repositories/helm-exporter/artifacts-tab/artifacts/sha256:98a69bbafd7c6d83ff12c7e70d6917be9970a8b19a8ad28d4d5f93333766d9e3</t>

</xml_diff>